<commit_message>
Corrections suite à la revue 7ad5e0697a0a9895ddcf8c15c2c3563456cc8364
</commit_message>
<xml_diff>
--- a/SBM-initDocIG/ig/StructureDefinition-fr-core-author.xlsx
+++ b/SBM-initDocIG/ig/StructureDefinition-fr-core-author.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-05T15:17:43+00:00</t>
+    <t>2025-02-05T15:35:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -417,7 +417,7 @@
 </t>
   </si>
   <si>
-    <t>Rôle fonctionnel de l'auteur. A utiliser uniquement si l'auteur est un professionnel.</t>
+    <t>Rôle fonctionnel de l'auteur.</t>
   </si>
   <si>
     <t>Author.functionCode.nullFlavor</t>

</xml_diff>